<commit_message>
Fix electricity connections + CO2 pipeline routes based on 5-closest rule
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/nodes/nodes.xlsx
+++ b/dac_offshore/clean_data/nodes/nodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\PycharmProjects\AdOpT_DAC-Offshore\dac_offshore\clean_data\nodes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/nodes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D54304-BE54-40EE-B7D9-95D682F338E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D17B14E-993D-9948-A6B2-D32260232555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2040" sheetId="1" r:id="rId1"/>
@@ -590,12 +590,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -618,7 +618,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -641,7 +641,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -664,7 +664,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -687,7 +687,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -710,7 +710,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -733,7 +733,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -756,7 +756,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -779,7 +779,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -802,7 +802,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -825,7 +825,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -848,7 +848,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -871,7 +871,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -894,7 +894,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -917,7 +917,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -940,7 +940,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -963,7 +963,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -986,7 +986,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1009,7 +1009,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>56</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>60</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>62</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>64</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -1400,7 +1400,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -1456,11 +1456,11 @@
       <c r="C38" t="s">
         <v>47</v>
       </c>
-      <c r="D38" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E38" t="e">
-        <v>#N/A</v>
+      <c r="D38">
+        <v>4.67</v>
+      </c>
+      <c r="E38">
+        <v>56.35</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -1469,7 +1469,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -1479,11 +1479,11 @@
       <c r="C39" t="s">
         <v>49</v>
       </c>
-      <c r="D39" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E39" t="e">
-        <v>#N/A</v>
+      <c r="D39">
+        <v>3.16</v>
+      </c>
+      <c r="E39">
+        <v>60.46</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -1492,7 +1492,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -1502,11 +1502,11 @@
       <c r="C40" t="s">
         <v>49</v>
       </c>
-      <c r="D40" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E40" t="e">
-        <v>#N/A</v>
+      <c r="D40">
+        <v>1.9</v>
+      </c>
+      <c r="E40">
+        <v>58.35</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1515,7 +1515,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>7</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -1607,7 +1607,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>5</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>10</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>16</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>15</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>2</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
NO_D coordinates fix. Added pipeline connections, fixed distances. Closes issue #35
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/nodes/nodes.xlsx
+++ b/dac_offshore/clean_data/nodes/nodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/nodes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/8051917/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/nodes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D17B14E-993D-9948-A6B2-D32260232555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA857BB-C0DE-144F-BB22-44CB4615C5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2040" sheetId="1" r:id="rId1"/>
@@ -1227,10 +1227,10 @@
         <v>49</v>
       </c>
       <c r="D28">
-        <v>25.641999999999999</v>
+        <v>21</v>
       </c>
       <c r="E28">
-        <v>71.424999999999997</v>
+        <v>71.599999999999994</v>
       </c>
       <c r="F28">
         <v>0</v>

</xml_diff>